<commit_message>
vata vizs moved to main.ipynb
</commit_message>
<xml_diff>
--- a/subsets.xlsx
+++ b/subsets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bruger\miniconda3\Lib\site-packages\my_folder\project-milestone-p2-group13\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F18266D-B6F6-4EC0-B369-3E792A78727A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0B351E-97AA-4A5E-91C1-4D7E15357737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="1" xr2:uid="{B0A9B495-6E7D-4A92-8DBB-0F9E53A28C0C}"/>
+    <workbookView xWindow="1830" yWindow="1830" windowWidth="17280" windowHeight="8904" activeTab="1" xr2:uid="{B0A9B495-6E7D-4A92-8DBB-0F9E53A28C0C}"/>
   </bookViews>
   <sheets>
     <sheet name="Train" sheetId="3" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="31">
   <si>
     <t>relationships</t>
   </si>
@@ -816,7 +816,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17F3EB24-4874-4781-93D3-5284019690AB}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="15.7890625" customWidth="1"/>
@@ -824,119 +824,119 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1">
-        <v>3539</v>
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B2">
-        <v>893</v>
+        <v>3539</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>472</v>
+        <v>893</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B4">
-        <v>417</v>
+        <v>472</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B5">
-        <v>161</v>
+        <v>417</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>132</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="B7">
-        <v>123</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B8">
-        <v>94</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B9">
-        <v>84</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B10">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="B11">
-        <v>60</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B12">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B13">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B14">
-        <v>39</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B15">
         <v>39</v>
@@ -944,31 +944,31 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B16">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B17">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="B18">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B19">
         <v>29</v>
@@ -976,31 +976,31 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B20">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B21">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B22">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>23</v>
@@ -1008,23 +1008,23 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B24">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="B25">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B26">
         <v>18</v>
@@ -1032,37 +1032,42 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B27">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B28">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
+        <v>17</v>
+      </c>
+      <c r="B29">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" t="s">
         <v>24</v>
       </c>
-      <c r="B29">
+      <c r="B30">
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="B30" s="1">
-        <f>SUM(B1:B29)</f>
-        <v>6553</v>
-      </c>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="B31" s="1"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B29">
-    <sortCondition descending="1" ref="B1:B29"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B30">
+    <sortCondition descending="1" ref="B2:B30"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1070,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43FF2A9-280C-49A3-AB0B-5BF9C251EE30}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="17.734375" customWidth="1"/>
@@ -1078,103 +1083,103 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1">
-        <v>3462</v>
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B2">
-        <v>891</v>
+        <v>3462</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>478</v>
+        <v>891</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B4">
-        <v>421</v>
+        <v>478</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B5">
-        <v>160</v>
+        <v>421</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>139</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B7">
-        <v>119</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B8">
-        <v>109</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B9">
-        <v>78</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="B10">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B11">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="B12">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>52</v>
@@ -1182,23 +1187,23 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B14">
-        <v>35</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B15">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="B16">
         <v>34</v>
@@ -1206,23 +1211,23 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B17">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B18">
-        <v>23</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B19">
         <v>23</v>
@@ -1230,23 +1235,23 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="B20">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="B21">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B22">
         <v>21</v>
@@ -1254,23 +1259,23 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B23">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B24">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B25">
         <v>19</v>
@@ -1278,7 +1283,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B26">
         <v>19</v>
@@ -1286,37 +1291,42 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B27">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="B28">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A30" t="s">
         <v>24</v>
       </c>
-      <c r="B29">
+      <c r="B30">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.55000000000000004">
-      <c r="B30" s="1">
-        <f>SUM(B1:B29)</f>
-        <v>6447</v>
-      </c>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.55000000000000004">
+      <c r="B31" s="1"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B29">
-    <sortCondition descending="1" ref="B1:B29"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B30">
+    <sortCondition descending="1" ref="B2:B30"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>